<commit_message>
feat(F-NAR-019): ATOM-COL.ECO.002-03 Le chat du carton
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.ECO.002-03.xlsx
+++ b/stories/arbres/ATOM-COL.ECO.002-03.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le fromage de la montagne</t>
+          <t>Le chat du carton</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>hall du marché, paille, fromage, carton de lait</t>
+          <t>cuisine à la farine, classe au tapis de pois, puis table</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Mila, maman</t>
+          <t>Mila, papa, maman, maîtresse</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Mila veut un bout du fromage qui sent la montagne. Elle parle trop tôt. Les voix du hall couvrent. Elle lève la main, elle attend, puis maman l'entend.</t>
+          <t>Mila veut dire le chat du carton. Un éclat de carton brille au coin plié. Elle coupe papa : les mots se perdent. À l'école, une voix trop près ; elle coupe, trop vite. Elle refuse de foncer, attend, raconte. Merci vécu. L'éclat de carton tient le gris.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le hall du marché sent le fromage chaud. De la paille craque sous les caisses. Un carton de lait a un chat gris. Les voix montent sous le toit de verre. Une cloche de fromage luit, toute ronde. Tu as senti, Mila ? Ça sent la montagne. Je veux un bout. On va le dire, alors. En ce moment, maman parle vers la cloche. Sa voix se mêle aux autres voix. Mila a les mots tout prêts. Un bout ! Celui qui sent la montagne ! Les mots tombent sous le toit de verre. Personne ne se tourne. La cloche reste loin, derrière la paille. Maman. Maman parle encore, un doigt vers le tarif. Mila ferme la bouche. Elle lève la main, tout droit. Sa main reste en l'air, près du carton. Le chat gris du carton la regarde. Une voix s'arrête, puis une autre. Maman se tourne. Tu voulais dire quelque chose ? Un bout. Celui qui sent la montagne. Je t'entends, maintenant. Un petit triangle blanc arrive dans un papier. Il est frais, un peu gras. C'est lui. Merci, Mila. Tu as attendu, et je t'ai entendue. Mila tient le papier à deux mains. Ça sent le lait et l'herbe sèche. On goûte sur le banc, dehors ? Oui.</t>
+          <t>La table en bois porte un voile blanc. C'est de la farine, froide sous le doigt. Un carton de lait se tient près du bol. Dessus, un chat gris lève le menton. Les moustaches dépassent, trop longues. Sur le coin plié, un éclat de carton brille. Il brille, maman ! Tu le vois, toi ? Oui, près des moustaches. Le lait est prêt, Mila. Ça sent le lait tiède, près du bol. Une fumée fine danse au-dessus. Le chat du carton est gris. Je veux le dire à l'école. On part après le bol ? Maintenant ! En ce moment, Mila coupe la phrase de papa. Les moustaches sont trop longues ! Les deux voix se cognent. Tu disais, Mila ? Le chat. Personne n'a la phrase entière. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Papa s'accroupit à la même hauteur. Tu veux parler, ou regarder le chat ? Parler. La boîte du goûter est prête. Mila glisse une pomme dans la boîte. Le cartable sent le cahier neuf. Les chaussures attendent près de la porte. Au revoir, papa. Tu dis bonjour, là-bas ? Oui, papa. Ta main est toute petite dans la mienne. Tu vas t'asseoir sur le tapis ? Oui, maman. Dans la rue, une sonnette de vélo tinte. Plus tard, l'école sent la craie. Les cahiers tapent un peu, dans le casier. Bonjour. Bonjour, maîtresse. Mila s'assoit sur le tapis. Le tapis a des pois verts. Un pois est un peu défait. Une image montre un chat gris. Les moustaches sont trop longues. C'est le même ! Les mots lui chatouillent la bouche. Elle veut le dire, ce chat, maintenant. Une voix s'approche, trop près. La voix veut le chat, elle aussi. Attends, je dois parler ! Ses mots se cognent à la voix. Mila referme la bouche. Les mains restent à plat sur ses genoux. Je veux parler du chat du lait.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le hall du marché sent le fromage chaud. De la paille craque sous les caisses. Un carton de lait a un chat gris. Les voix montent sous le toit de verre. Une cloche de fromage luit, toute ronde. Tu as senti, Mila ? Ça sent la montagne. Je veux un bout. On va le dire, alors. En ce moment, maman parle vers la cloche. Sa voix se mêle aux autres voix. Mila a les mots tout prêts. Un bout ! Celui qui sent la montagne ! Les mots tombent sous le toit de verre. Personne ne se tourne. La cloche reste loin, derrière la paille. Maman. Maman parle encore, un doigt vers le tarif. Mila ferme la bouche. Elle lève la main, tout droit. Sa main reste en l'air, près du carton. Le chat gris du carton la regarde. Une voix s'arrête, puis une autre. Maman se tourne. Tu voulais dire quelque chose ? Un bout. Celui qui sent la montagne. Je t'entends, maintenant. Un petit triangle blanc arrive dans un papier. Il est frais, un peu gras. C'est lui. Merci, Mila. Tu as attendu, et je t'ai entendue. Mila tient le papier à deux mains. Ça sent le lait et l'herbe sèche. On goûte sur le banc, dehors ? Oui.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La table en bois porte un voile blanc. C'est de la farine, froide sous le doigt. Un carton de lait se tient près du bol. Dessus, un chat gris lève le menton. Les moustaches dépassent, trop longues. Sur le coin plié, un &lt;emphasis level="moderate"&gt;éclat de carton&lt;/emphasis&gt; brille. Il brille, maman ! Tu le vois, toi ? Oui, près des moustaches. Le lait est prêt, Mila. Ça sent le lait tiède, près du bol. Une fumée fine danse au-dessus. Le chat du carton est gris. Je veux le dire à l'école. On part après le bol ? Maintenant ! En ce moment, Mila coupe la phrase de papa. Les moustaches sont trop longues ! Les deux voix se cognent. Tu disais, Mila ? Le chat. Personne n'a la phrase entière. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Papa s'accroupit à la même hauteur. Tu veux parler, ou regarder le chat ? Parler. La boîte du goûter est prête. Mila glisse une pomme dans la boîte. Le cartable sent le cahier neuf. Les chaussures attendent près de la porte. Au revoir, papa. Tu dis bonjour, là-bas ? Oui, papa. Ta main est toute petite dans la mienne. Tu vas t'asseoir sur le tapis ? Oui, maman. Dans la rue, une sonnette de vélo tinte. Plus tard, l'école sent la craie. Les cahiers tapent un peu, dans le casier. Bonjour. Bonjour, maîtresse. Mila s'assoit sur le tapis. Le tapis a des pois verts. Un pois est un peu défait. Une image montre un chat gris. Les moustaches sont trop longues. C'est le même ! Les mots lui chatouillent la bouche. Elle veut le dire, ce chat, maintenant. Une voix s'approche, trop près. La voix veut le chat, elle aussi. Attends, je dois parler ! Ses mots se cognent à la voix. Mila referme la bouche. Les mains restent à plat sur ses genoux. Je veux parler du chat du lait.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Fatou arrive en classe avec maman. Maman dit au revoir. Fatou s'assoit sur le tapis. La maîtresse pose une question. Fatou a une idée. Elle lève la main. Il faut &lt;emphasis&gt;attendre&lt;/emphasis&gt;. Un camarade parle d'abord. Fatou attend encore. Puis la maîtresse dit : Fatou, c'est ton tour. Fatou parle. Elle dit : le chat est gris. La maîtresse sourit. Le soir, à table, papa pose une question. Fatou se souvient. Elle lève la main. Papa sourit. Il faut attendre. Papa écoute maman d'abord. Fatou attend. Puis papa dit : Fatou, c'est toi. Fatou parle. Elle raconte le chat gris. Maman demande. Fatou dit : j'ai levé la main. J'ai su attendre. Puis parler. Papa dit : merci. Le tour de parole, c'est à l'école et à la maison. [pause]</t>
+          <t>La table en bois porte un voile blanc. C'est de la farine, froide sous le doigt. Un carton de lait se tient près du bol. Dessus, un chat gris lève le menton. Les moustaches dépassent, trop longues. Sur le coin plié, un &lt;emphasis&gt;éclat de carton&lt;/emphasis&gt; brille. Il brille, maman ! Tu le vois, toi ? Oui, près des moustaches. Le lait est prêt, Mila. Ça sent le lait tiède, près du bol. Une fumée fine danse au-dessus. Le chat du carton est gris. Je veux le dire à l'école. On part après le bol ? Maintenant ! En ce moment, Mila coupe la phrase de papa. Les moustaches sont trop longues ! Les deux voix se cognent. Tu disais, Mila ? Le chat. Personne n'a la phrase entière. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Papa s'accroupit à la même hauteur. Tu veux parler, ou regarder le chat ? Parler. La boîte du goûter est prête. Mila glisse une pomme dans la boîte. Le cartable sent le cahier neuf. Les chaussures attendent près de la porte. Au revoir, papa. Tu dis bonjour, là-bas ? Oui, papa. Ta main est toute petite dans la mienne. Tu vas t'asseoir sur le tapis ? Oui, maman. Dans la rue, une sonnette de vélo tinte. Plus tard, l'école sent la craie. Les cahiers tapent un peu, dans le casier. Bonjour. Bonjour, maîtresse. Mila s'assoit sur le tapis. Le tapis a des pois verts. Un pois est un peu défait. Une image montre un chat gris. Les moustaches sont trop longues. C'est le même ! Les mots lui chatouillent la bouche. Elle veut le dire, ce chat, maintenant. Une voix s'approche, trop près. La voix veut le chat, elle aussi. Attends, je dois parler ! Ses mots se cognent à la voix. Mila referme la bouche. Les mains restent à plat sur ses genoux. Je veux parler du chat du lait. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>attendre</t>
+          <t>éclat de carton</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,47 +1326,70 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse; intensite=2; destinataire=enfant; sous_texte=l_eclat_de_carton_au_coin_plie; tempo=naturel; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le hall du marché sent le fromage chaud.
-narrateur|De la paille craque sous les caisses.
-narrateur|Un carton de lait a un chat gris.
-narrateur|Les voix montent sous le toit de verre.
-narrateur|Une cloche de fromage luit, toute ronde.
-maman|Tu as senti, Mila ?
-enfant-f|Ça sent la montagne.
-enfant-f|Je veux un bout.
-maman|On va le dire, alors.
-narrateur|En ce moment, maman parle vers la cloche.
-narrateur|Sa voix se mêle aux autres voix.
-narrateur|Mila a les mots tout prêts.
-enfant-f|Un bout !
-enfant-f|Celui qui sent la montagne !
-narrateur|Les mots tombent sous le toit de verre.
-narrateur|Personne ne se tourne.
-narrateur|La cloche reste loin, derrière la paille.
-enfant-f|Maman.
-narrateur|Maman parle encore, un doigt vers le tarif.
-narrateur|Mila ferme la bouche.
-narrateur|Elle lève la main, tout droit.
-narrateur|Sa main reste en l'air, près du carton.
-narrateur|Le chat gris du carton la regarde.
-narrateur|Une voix s'arrête, puis une autre.
-narrateur|Maman se tourne.
-maman|Tu voulais dire quelque chose ?
-enfant-f|Un bout.
-enfant-f|Celui qui sent la montagne.
-maman|Je t'entends, maintenant.
-narrateur|Un petit triangle blanc arrive dans un papier.
-narrateur|Il est frais, un peu gras.
-enfant-f|C'est lui.
-maman|Merci, Mila.
-maman|Tu as attendu, et je t'ai entendue.
-narrateur|Mila tient le papier à deux mains.
-narrateur|Ça sent le lait et l'herbe sèche.
-maman|On goûte sur le banc, dehors ?
-enfant-f|Oui.</t>
+          <t>narrateur|La table en bois porte un voile blanc.
+narrateur|C'est de la farine, froide sous le doigt.
+narrateur|Un carton de lait se tient près du bol.
+narrateur|Dessus, un chat gris lève le menton.
+narrateur|Les moustaches dépassent, trop longues.
+narrateur|Sur le coin plié, un éclat de carton brille.
+enfant-f|Il brille, maman !
+maman|Tu le vois, toi ?
+enfant-f|Oui, près des moustaches.
+papa|Le lait est prêt, Mila.
+narrateur|Ça sent le lait tiède, près du bol.
+narrateur|Une fumée fine danse au-dessus.
+enfant-f|Le chat du carton est gris.
+enfant-f|Je veux le dire à l'école.
+papa|On part après le bol ?
+enfant-f|Maintenant !
+narrateur|En ce moment, Mila coupe la phrase de papa.
+enfant-f|Les moustaches sont trop longues !
+narrateur|Les deux voix se cognent.
+papa|Tu disais, Mila ?
+enfant-f|Le chat.
+narrateur|Personne n'a la phrase entière.
+narrateur|Le sourire de Mila disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu veux parler, ou regarder le chat ?
+enfant-f|Parler.
+maman|La boîte du goûter est prête.
+narrateur|Mila glisse une pomme dans la boîte.
+narrateur|Le cartable sent le cahier neuf.
+narrateur|Les chaussures attendent près de la porte.
+enfant-f|Au revoir, papa.
+papa|Tu dis bonjour, là-bas ?
+enfant-f|Oui, papa.
+maman|Ta main est toute petite dans la mienne.
+maman|Tu vas t'asseoir sur le tapis ?
+enfant-f|Oui, maman.
+narrateur|Dans la rue, une sonnette de vélo tinte.
+narrateur|Plus tard, l'école sent la craie.
+narrateur|Les cahiers tapent un peu, dans le casier.
+maitresse|Bonjour.
+enfant-f|Bonjour, maîtresse.
+narrateur|Mila s'assoit sur le tapis.
+narrateur|Le tapis a des pois verts.
+narrateur|Un pois est un peu défait.
+narrateur|Une image montre un chat gris.
+narrateur|Les moustaches sont trop longues.
+enfant-f|C'est le même !
+narrateur|Les mots lui chatouillent la bouche.
+narrateur|Elle veut le dire, ce chat, maintenant.
+narrateur|Une voix s'approche, trop près.
+narrateur|La voix veut le chat, elle aussi.
+enfant-f|Attends, je dois parler !
+narrateur|Ses mots se cognent à la voix.
+narrateur|Mila referme la bouche.
+narrateur|Les mains restent à plat sur ses genoux.
+enfant-f|Je veux parler du chat du lait.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1403,12 +1426,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Mila veut parler. Que fait-elle d'abord ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Mila veut parler. Que fait-elle &lt;emphasis level="moderate"&gt;d'abord&lt;/emphasis&gt; ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Fatou veut parler. Que fait-elle d'abord ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Mila veut parler. Que fait-elle &lt;emphasis&gt;d'abord&lt;/emphasis&gt; ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1471,7 +1494,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1479,10 +1502,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1497,34 +1520,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>d'abord</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1533,23 +1560,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_attend_avant_de_parler; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1582,17 +1609,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Le banc dehors est tiède. Mila ouvre le papier. Le triangle a des petits trous. Ça sent vraiment la montagne. Tu croques ? Oui. Le fromage est doux, un peu piquant. Tu m'as entendue. Oui. Quand les voix se sont tues un peu. Quand ta main était là. Le carton de lait est dans le cabas. Le chat gris les regarde encore. Il te plaît, le chat ? Il a des moustaches trop longues. Mila lèche un peu de gras au pouce. Le papier craque, tout léger. Il en reste ? Un tout petit bout.</t>
+          <t>Mila lève la main. Sa main reste en l'air. Les doigts tremblent un peu. Une autre voix parle d'abord. On entend parler des moustaches. Mila garde la main levée. Mila ? Mila parle. Le chat est gris. Comme le chat du carton, à la maison. Les mots arrivent entiers, cette fois. Le soir, les assiettes sont chaudes. Ça sent le gratin. La nappe a des petits carreaux. Alors, Mila ? Mila sent l'envie revenir. Elle lève la main, même à table. Papa écoute maman d'abord. Le gratin est prêt. Mila attend que le silence arrive. Elle pose l'autre main sur la nappe. Mila, c'est toi. Le chat de l'école est le même. Il est sur le carton. Merci de nous le dire, Mila. Papa a entendu toute la phrase. Le ventre de Mila se desserre. Sur le carton, l'éclat de carton revient. Tu as soif ? Un peu. Mila prend une gorgée. L'eau chante contre le verre. C'est frais.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Le banc dehors est tiède. Mila ouvre le papier. Le triangle a des petits trous. Ça sent vraiment la montagne. Tu croques ? Oui. Le fromage est doux, un peu piquant. Tu m'as entendue. Oui. Quand les voix se sont tues un peu. Quand ta main était là. Le carton de lait est dans le cabas. Le chat gris les regarde encore. Il te plaît, le chat ? Il a des moustaches trop longues. Mila lèche un peu de gras au pouce. Le papier craque, tout léger. Il en reste ? Un tout petit bout.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila lève la main. Sa main reste en l'air. Les doigts tremblent un peu. Une autre voix parle d'abord. On entend parler des moustaches. Mila garde la main levée. Mila ? Mila parle. Le chat est gris. Comme le chat du carton, à la maison. Les mots arrivent entiers, cette fois. Le soir, les assiettes sont chaudes. Ça sent le gratin. La nappe a des petits carreaux. Alors, Mila ? Mila sent l'envie revenir. Elle lève la main, même à table. Papa écoute maman d'abord. Le gratin est prêt. Mila attend que le silence arrive. Elle pose l'autre main sur la nappe. Mila, c'est toi. Le chat de l'école est le même. Il est sur le carton. Merci de nous le dire, Mila. Papa a entendu toute la phrase. Le ventre de Mila se desserre. Sur le carton, l'&lt;emphasis level="moderate"&gt;éclat de carton&lt;/emphasis&gt; revient. Tu as soif ? Un peu. Mila prend une gorgée. L'eau chante contre le verre. C'est frais.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Fatou a levé la main. Elle a attendu. &lt;emphasis&gt;puis&lt;/emphasis&gt; parler, c'était son tour. À l'école et à table. [pause]</t>
+          <t>Mila lève la main. Sa main reste en l'air. Les doigts tremblent un peu. Une autre voix parle d'abord. On entend parler des moustaches. Mila garde la main levée. Mila ? Mila parle. Le chat est gris. Comme le chat du carton, à la maison. Les mots arrivent entiers, cette fois. Le soir, les assiettes sont chaudes. Ça sent le gratin. La nappe a des petits carreaux. Alors, Mila ? Mila sent l'envie revenir. Elle lève la main, même à table. Papa écoute maman d'abord. Le gratin est prêt. Mila attend que le silence arrive. Elle pose l'autre main sur la nappe. Mila, c'est toi. Le chat de l'école est le même. Il est sur le carton. Merci de nous le dire, Mila. Papa a entendu toute la phrase. Le ventre de Mila se desserre. Sur le carton, l'&lt;emphasis&gt;éclat de carton&lt;/emphasis&gt; revient. Tu as soif ? Un peu. Mila prend une gorgée. L'eau chante contre le verre. C'est frais. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1639,7 +1666,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1647,10 +1674,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1673,30 +1700,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>puis</t>
+          <t>éclat de carton</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1705,10 +1732,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1721,30 +1748,44 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_attend_puis_on_l_entend; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Le banc dehors est tiède.
-narrateur|Mila ouvre le papier.
-narrateur|Le triangle a des petits trous.
-enfant-f|Ça sent vraiment la montagne.
-maman|Tu croques ?
-enfant-f|Oui.
-narrateur|Le fromage est doux, un peu piquant.
-enfant-f|Tu m'as entendue.
-maman|Oui.
-maman|Quand les voix se sont tues un peu.
-maman|Quand ta main était là.
-narrateur|Le carton de lait est dans le cabas.
-narrateur|Le chat gris les regarde encore.
-maman|Il te plaît, le chat ?
-enfant-f|Il a des moustaches trop longues.
-narrateur|Mila lèche un peu de gras au pouce.
-narrateur|Le papier craque, tout léger.
-maman|Il en reste ?
-enfant-f|Un tout petit bout.</t>
+          <t>narrateur|Mila lève la main.
+narrateur|Sa main reste en l'air.
+narrateur|Les doigts tremblent un peu.
+narrateur|Une autre voix parle d'abord.
+narrateur|On entend parler des moustaches.
+narrateur|Mila garde la main levée.
+maitresse|Mila ?
+narrateur|Mila parle.
+enfant-f|Le chat est gris.
+enfant-f|Comme le chat du carton, à la maison.
+narrateur|Les mots arrivent entiers, cette fois.
+narrateur|Le soir, les assiettes sont chaudes.
+narrateur|Ça sent le gratin.
+narrateur|La nappe a des petits carreaux.
+papa|Alors, Mila ?
+narrateur|Mila sent l'envie revenir.
+narrateur|Elle lève la main, même à table.
+narrateur|Papa écoute maman d'abord.
+maman|Le gratin est prêt.
+narrateur|Mila attend que le silence arrive.
+narrateur|Elle pose l'autre main sur la nappe.
+papa|Mila, c'est toi.
+enfant-f|Le chat de l'école est le même.
+enfant-f|Il est sur le carton.
+maman|Merci de nous le dire, Mila.
+narrateur|Papa a entendu toute la phrase.
+narrateur|Le ventre de Mila se desserre.
+narrateur|Sur le carton, l'éclat de carton revient.
+papa|Tu as soif ?
+enfant-f|Un peu.
+narrateur|Mila prend une gorgée.
+narrateur|L'eau chante contre le verre.
+enfant-f|C'est frais.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
@@ -1776,17 +1817,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Maman plie le papier vide. Il sent encore la montagne. On rentre ? Oui. J'ai eu mon bout. Oui. Je t'ai entendue. Le hall rumine, plus loin, plus bas. La paille reste collée à une chaussure. Tu la secoues ? Oui, maman.</t>
+          <t>Mila glisse de la chaise. Le chat, je le montre ! Elle court vers le carton. Elle le tourne d'un grand geste. Le coin plié se cache. L'éclat de carton n'est plus là. Il est parti ! Le sourire tremble. Tu le cherches ? Oui. Mila refuse de foncer. Elle reste près du carton. Personne ne parle. Ses doigts attendent sur le bois. Elle tourne le carton, sans se presser. Le coin plié revient vers la lampe. Comme ce matin ! Tu le vois, toi ? Mila pose un doigt, sans frotter. L'éclat de carton saute près des moustaches. Il est revenu. Il m'a attendue. La table garde le gratin.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Maman plie le papier vide. Il sent encore la montagne. On rentre ? Oui. J'ai eu mon bout. Oui. Je t'ai entendue. Le hall rumine, plus loin, plus bas. La paille reste collée à une chaussure. Tu la secoues ? Oui, maman.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Mila glisse de la chaise. Le chat, je le montre ! Elle court vers le carton. Elle le tourne d'un grand geste. Le coin plié se cache. L'&lt;emphasis level="moderate"&gt;éclat de carton&lt;/emphasis&gt; n'est plus là. Il est parti ! Le sourire tremble. Tu le cherches ? Oui. Mila refuse de foncer. Elle reste près du carton. Personne ne parle. Ses doigts attendent sur le bois. Elle tourne le carton, sans se presser. Le coin plié revient vers la lampe. Comme ce matin ! Tu le vois, toi ? Mila pose un doigt, sans frotter. L'éclat de carton saute près des moustaches. Il est revenu. Il m'a attendue. La table garde le gratin.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Fatou range son cartable. Maman l'attend à la porte. [pause]</t>
+          <t>&lt;low-pitch&gt;Mila glisse de la chaise. Le chat, je le montre ! Elle court vers le carton. Elle le tourne d'un grand geste. Le coin plié se cache. L'&lt;emphasis&gt;éclat de carton&lt;/emphasis&gt; n'est plus là. Il est parti ! Le sourire tremble. Tu le cherches ? Oui. Mila refuse de foncer. Elle reste près du carton. Personne ne parle. Ses doigts attendent sur le bois. Elle tourne le carton, sans se presser. Le coin plié revient vers la lampe. Comme ce matin ! Tu le vois, toi ? Mila pose un doigt, sans frotter. L'éclat de carton saute près des moustaches. Il est revenu. Il m'a attendue. La table garde le gratin.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1833,7 +1874,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1841,22 +1882,26 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1865,28 +1910,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de carton</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1895,34 +1944,50 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=deux_envies_qui_se_heurtent; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_retrouve_l_eclat_de_carton; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Maman plie le papier vide.
-narrateur|Il sent encore la montagne.
-maman|On rentre ?
+          <t>narrateur|Mila glisse de la chaise.
+enfant-f|Le chat, je le montre !
+narrateur|Elle court vers le carton.
+narrateur|Elle le tourne d'un grand geste.
+narrateur|Le coin plié se cache.
+narrateur|L'éclat de carton n'est plus là.
+enfant-f|Il est parti !
+narrateur|Le sourire tremble.
+papa|Tu le cherches ?
 enfant-f|Oui.
-enfant-f|J'ai eu mon bout.
-maman|Oui.
-maman|Je t'ai entendue.
-narrateur|Le hall rumine, plus loin, plus bas.
-narrateur|La paille reste collée à une chaussure.
-maman|Tu la secoues ?
-enfant-f|Oui, maman.</t>
+narrateur|Mila refuse de foncer.
+narrateur|Elle reste près du carton.
+narrateur|Personne ne parle.
+narrateur|Ses doigts attendent sur le bois.
+narrateur|Elle tourne le carton, sans se presser.
+narrateur|Le coin plié revient vers la lampe.
+enfant-f|Comme ce matin !
+maman|Tu le vois, toi ?
+narrateur|Mila pose un doigt, sans frotter.
+narrateur|L'éclat de carton saute près des moustaches.
+papa|Il est revenu.
+enfant-f|Il m'a attendue.
+narrateur|La table garde le gratin.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
@@ -1954,17 +2019,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le papier vide sent encore le lait. Tu m'as entendue. Oui. Le chat gris reste sur le carton. Le hall est loin, maintenant.</t>
+          <t>Maman tourne le carton de lait. Le chat gris les regarde. C'est lui. On reste un peu ? Oui, maman. Mila serre le bol contre elle. Le lait n'est plus tiède. On se dit bonne nuit dans un moment ? Oui, papa. Le cartable sent la farine du matin. Il est là. On le garde des yeux ? Oui. L'éclat de carton tient le gris.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le papier vide sent encore le lait. Tu m'as entendue. Oui. Le chat gris reste sur le carton. Le hall est loin, maintenant.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Maman tourne le carton de lait. Le chat gris les regarde. C'est lui. On reste un peu ? Oui, maman. Mila serre le bol contre elle. Le lait n'est plus tiède. On se dit bonne nuit dans un moment ? Oui, papa. Le cartable sent la farine du matin. Il est là. On le garde des yeux ? Oui. L'&lt;emphasis level="moderate"&gt;éclat de carton&lt;/emphasis&gt; tient le gris.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Maman tourne le carton de lait. Le chat gris les regarde. C'est lui. On reste un peu ? Oui, maman. Mila serre le bol contre elle. Le lait n'est plus tiède. On se dit bonne nuit dans un moment ? Oui, papa. Le cartable sent la farine du matin. Il est là. On le garde des yeux ? Oui. L'&lt;emphasis&gt;éclat de carton&lt;/emphasis&gt; tient le gris.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2011,18 +2076,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2031,12 +2096,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2045,17 +2110,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de carton</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2064,11 +2133,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2077,28 +2146,41 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_de_carton_tient_le_gris; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le papier vide sent encore le lait.
-enfant-f|Tu m'as entendue.
-maman|Oui.
-narrateur|Le chat gris reste sur le carton.
-narrateur|Le hall est loin, maintenant.</t>
+          <t>narrateur|Maman tourne le carton de lait.
+narrateur|Le chat gris les regarde.
+enfant-f|C'est lui.
+maman|On reste un peu ?
+enfant-f|Oui, maman.
+narrateur|Mila serre le bol contre elle.
+narrateur|Le lait n'est plus tiède.
+papa|On se dit bonne nuit dans un moment ?
+enfant-f|Oui, papa.
+narrateur|Le cartable sent la farine du matin.
+enfant-f|Il est là.
+maman|On le garde des yeux ?
+enfant-f|Oui.
+narrateur|L'éclat de carton tient le gris.</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2201,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2211,6 +2293,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>